<commit_message>
Coverage and SSN issue solved
</commit_message>
<xml_diff>
--- a/Unified_PDF_Platform/unified_outputs/APL- Rapid Trading- Dec 25_invoice.xlsx
+++ b/Unified_PDF_Platform/unified_outputs/APL- Rapid Trading- Dec 25_invoice.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -547,22 +547,22 @@
           <t>1560</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2480131</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2480131</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
         <v>61.34</v>
@@ -588,7 +588,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -607,22 +607,22 @@
           <t>8855</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2480128</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2480128</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>128.93</v>
@@ -648,7 +648,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -667,22 +667,22 @@
           <t>1486</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2480132</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2480132</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
         <v>101.85</v>
@@ -708,7 +708,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -727,22 +727,22 @@
           <t>4279</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2480130</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2480130</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
         <v>61.34</v>
@@ -768,7 +768,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -787,22 +787,22 @@
           <t>9511</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2480129</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2480129</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>61.34</v>
@@ -828,7 +828,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -847,22 +847,22 @@
           <t>5214</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2480127</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2480127</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
         <v>128.93</v>
@@ -888,7 +888,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -907,22 +907,22 @@
           <t>0016</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2559492</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2559492</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
         <v>61.34</v>
@@ -948,7 +948,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>202512</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -967,22 +967,22 @@
           <t>3439</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2480133</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>MEDLINK9 GROUP MED SUP</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2480133</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>MEDLINK9 GROUP MED SUP</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>MEDICAL</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
         <v>61.34</v>

</xml_diff>